<commit_message>
feat: live quote verification pipeline, price change detection, and updated master catalog
</commit_message>
<xml_diff>
--- a/master_catalog.xlsx
+++ b/master_catalog.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T12:56:26.274973+00:00</t>
+          <t>2026-10-17T13:13:42.740440+00:00</t>
         </is>
       </c>
     </row>
@@ -579,15 +579,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -843,6 +843,286 @@
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>INSPECT_PUBLIC_URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/s/premiumtoolschat</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/spaivault_bot</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/s/ptsbd26</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/MediaHubMarketplace_bot</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/s/mmoglobalhub</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/prmastbot</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/s/toolorax</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/s/sealsareana</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/FatBunny_Hub_bot</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>INTERACTIVE_MENU_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Bot requires interactive chat and /start command. Automated scraping without user session not permitted.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Review catalog via Telegram app and record quote using Streamlit Manual Entry</t>
         </is>
       </c>
     </row>
@@ -3934,7 +4214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3947,7 +4227,7 @@
     <col width="27" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="39" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5432,6 +5712,1995 @@
       <c r="K29" s="2" t="inlineStr">
         <is>
           <t>https://t.me/s/digicarttools</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>duolingo__duolingo_super_promo__12_months__promo_code</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>proton_vpn__proton_vpn_plus_1y__12_months__private</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>1271.25</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>autodesk__autodesk_all_apps_aec__3_years__edu</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>367.25</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>proton_vpn__proton_vpn_plus_lifetime__lifetime__private</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>2260</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>coursera__coursera_plus__12_months__private</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>988.75</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>ilovepdf__ilovepdf_premium__12_months__private</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>1130</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>1469</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>3531.25</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>jetbrains__jetbrains_all_products_pack__12_months__edu</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>1045.25</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>1356</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>2599</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>2260</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>5650</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>2260</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>DigiCart Tools</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>1412.5</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/digicarttools/20</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_student__4_months__edu</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>2497.3</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_edu__2_years__edu</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>1307.97</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>5h Warranty</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>netflix__netflix_4k_uhd_profile__1_month__shared</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>915.3</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>netflix__netflix_4k_uhd_profile_3m__3_months__shared</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>2152.65</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team__6_months__team</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>3480.4</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_student__4_months__edu</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>3042.53</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_personal__1_month__private</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>358.77</v>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>2152.65</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>1 Day Warranty</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_student__4_months__edu</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>3166.83</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12 UTC</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAIPremium/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>heygen__heygen_ai_avatar_creator__1_month__private</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Sellnity Store</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>3551.03</v>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>1 day Warranty</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/sellnitystoreupdates/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>krea_ai__krea_ai_basic__1_month__private</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Sellnity Store</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>1689.35</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>1 day Warranty</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/sellnitystoreupdates/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>kling_ai__kling_ai_video_standard__1_month__private</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Sellnity Store</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>1418.15</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/sellnitystoreupdates/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team__6_months__team</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Sellnity Store</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>3971.95</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/sellnitystoreupdates/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>autodesk__autodesk_all_apps_aec__3_years__edu</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Sellnity Store</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>8771.620000000001</v>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/sellnitystoreupdates/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>ilovepdf__ilovepdf_premium__12_months__private</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Sellnity Store</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>288.15</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/sellnitystoreupdates/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>leonardo_ai__leonardo_ai_essential__1_month__private</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>NovaShop Premium</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>282.5</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/novasubpre/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>NovaShop Premium</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>2960.6</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/novasubpre/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>NovaShop Premium</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>2960.6</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/novasubpre/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>NovaShop Premium</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>2960.6</v>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/novasubpre/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>google_gemini__gemini_pro_invitation__18_months__invite</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>AI Toolify</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>127.12</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/hacksxtips/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>google_gemini__gemini_pro_invitation__18_months__invite</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>AI Toolify</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>118.65</v>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>No Warranty (NW)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/hacksxtips/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>AI Toolify</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>28.25</v>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/hacksxtips/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>google_gemini__gemini_pro_invitation__18_months__invite</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Verified Streams</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>169.5</v>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/verifiedstreams/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>AIToolPre Bot</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>141250</v>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>3 days Warranty</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13 UTC</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/Airdrop_Crypto_x100/15</t>
         </is>
       </c>
     </row>
@@ -5525,28 +7794,28 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DigiCart Tools</t>
+          <t>AI Toolify</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USDT</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1400</v>
+        <v>28.25</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Full Warranty (FW)</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>USER_SUPPLIED_UNVERIFIED</t>
+          <t>Not Stated</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
         </is>
       </c>
     </row>
@@ -5959,32 +8228,28 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>No Verified Winner Yet</t>
+          <t>PiggyAI Premium</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>3480.4</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Full Warranty (FW)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>PENDING_QUOTES</t>
+          <t>VERIFIED</t>
         </is>
       </c>
     </row>
@@ -6565,32 +8830,28 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>No Verified Winner Yet</t>
+          <t>PiggyAI Premium</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>915.3</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Full Warranty (FW)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>PENDING_QUOTES</t>
+          <t>VERIFIED</t>
         </is>
       </c>
     </row>
@@ -6648,18 +8909,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6706,6 +8967,474 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $5.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $12.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_DROP</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $4.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $9.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $8.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $20.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus__1_month__private</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @digicarttools: $5.0 -&gt; $8.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_student__4_months__edu</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @PiggyAIPremium: $7.7 -&gt; $8.84</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>netflix__netflix_4k_uhd_profile_3m__3_months__shared</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @PiggyAIPremium: $3.24 -&gt; $7.62</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_student__4_months__edu</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @PiggyAIPremium: $7.7 -&gt; $10.77</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt__chatgpt_plus_student__4_months__edu</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:12</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @PiggyAIPremium: $7.7 -&gt; $11.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>google_gemini__gemini_pro_invitation__18_months__invite</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>PRICE_INCREASE</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:13</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Live public price change detected on @hacksxtips: $0.42 -&gt; $0.45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: ingest verified real bot quotes from user screen recording (HitMeow vs PiggyAI)
</commit_message>
<xml_diff>
--- a/master_catalog.xlsx
+++ b/master_catalog.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T13:13:42.740440+00:00</t>
+          <t>2026-10-17T13:45:16.613619+00:00</t>
         </is>
       </c>
     </row>
@@ -2620,12 +2620,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -3228,6 +3228,126 @@
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Entertainment &amp; Streaming</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Coding AI &amp; IDE</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>VPN &amp; Security</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Audio &amp; Voice AI</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3244,12 +3364,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -4200,6 +4320,636 @@
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>netflix__netflix_4k_uhd_profile_3m__3_months__shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>CapCut</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CapCut Pro Team 3 Months</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team__3_months__team</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium Slot 3 Months</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>youtube_premium__youtube_premium_slot_3_months__3_months__shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium Slot 6 Months</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>youtube_premium__youtube_premium_slot_6_months__6_months__shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium Slot 1 Year</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>youtube_premium__youtube_premium_slot_1_year__1_year__shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro API 2600 Credits 1M</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>cursor_pro__cursor_pro_api_2600_credits_1m__1_month__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro API 6500 Credits 1M</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>cursor_pro__cursor_pro_api_6500_credits_1m__1_month__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Claude API 50M Tokens 1D</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>1 Day</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_50m_tokens_1d__1_day__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Claude API 100M Tokens 1D</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>1 Day</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_100m_tokens_1d__1_day__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Claude API  Token 1M</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_token_1m__1_month__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Claude Kiro API  1M</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_kiro_api_1m__1_month__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Grok</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Grok API 10M Credit 1M</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Token</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>grok__grok_api_10m_credit_1m__1_month__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>CapCut</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>CapCut Pro Team 3 Months</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team_3_months__3_months__team</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>CapCut</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>CapCut Pro Personal 3 Months</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>PRIVATE</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_personal_3_months__3_months__private</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>CapCut</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>CapCut Pro Team 12 Months</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>12 Months</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team_12_months__12_months__team</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN 10 Devices 3M</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>nordvpn__nordvpn_10_devices_3m__3_months__shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN Slot 6M</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>nordvpn__nordvpn_slot_6m__6_months__shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro 2026 Credits 1M</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>cursor_pro__cursor_pro_2026_credits_1m__1_month__api</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs Redeem 100k Credits</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>elevenlabs__elevenlabs_redeem_100k_credits__1_month__key</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7704,6 +8454,1281 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team__3_months__team</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>1740.2</v>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>youtube_premium__youtube_premium_slot_3_months__3_months__shared</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>1028.3</v>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>youtube_premium__youtube_premium_slot_6_months__6_months__shared</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>1788.22</v>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>youtube_premium__youtube_premium_slot_1_year__1_year__shared</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>3031.22</v>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>cursor_pro__cursor_pro_api_2600_credits_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>2409.72</v>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>cursor_pro__cursor_pro_api_6500_credits_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>3401.3</v>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_50m_tokens_1d__1_day__api</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>601.73</v>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_100m_tokens_1d__1_day__api</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>1087.62</v>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_token_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>1517.03</v>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>30 Days Warranty</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_api_token_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>34.96</v>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>9876.200000000001</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_kiro_api_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>2491.65</v>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>claude__claude_kiro_api_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>3842</v>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>grok__grok_api_10m_credit_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>539.5700000000001</v>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26 UTC</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_personal__1_month__private</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>353.12</v>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_personal__1_month__private</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>358.77</v>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team_3_months__3_months__team</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>1740.2</v>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team_3_months__3_months__team</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>2056.6</v>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_personal_3_months__3_months__private</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>1056.55</v>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>capcut__capcut_pro_team_12_months__12_months__team</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>22.82</v>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>6446.65</v>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>nordvpn__nordvpn_10_devices_3m__3_months__shared</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>587.6</v>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>nordvpn__nordvpn_slot_6m__6_months__shared</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>1175.2</v>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>cursor_pro__cursor_pro_2026_credits_1m__1_month__api</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>2378.65</v>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>elevenlabs__elevenlabs_redeem_100k_credits__1_month__key</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>293.8</v>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>kling_ai__kling_ai_video_standard__1_month__private</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>1469</v>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PremiKeyBot</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>google_gemini__gemini_pro_invitation__18_months__invite</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>127.12</v>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>24H Warranty</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/PiggyAi799_Bot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7715,10 +9740,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
@@ -8185,28 +10210,28 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>PiggyAI Premium</t>
+          <t>PremiKey Bot</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USDT</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1.27</v>
+        <v>1.25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>355.6</v>
+        <v>353.12</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Working</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>USER_SUPPLIED_UNVERIFIED</t>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
         </is>
       </c>
     </row>
@@ -8895,6 +10920,780 @@
       <c r="I27" s="3" t="inlineStr">
         <is>
           <t>USER_SUPPLIED_UNVERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>CapCut - CapCut Pro Team 3 Months</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1740.2</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium - YouTube Premium Slot 3 Months</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>1028.3</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium - YouTube Premium Slot 6 Months</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>1788.22</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>YouTube Premium - YouTube Premium Slot 1 Year</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>3031.22</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro - Cursor Pro API 2600 Credits 1M</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>2409.72</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro - Cursor Pro API 6500 Credits 1M</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>3401.3</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Claude - Claude API 50M Tokens 1D</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>1 Day</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>601.73</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Claude - Claude API 100M Tokens 1D</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>1 Day</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>1087.62</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Claude - Claude API  Token 1M</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>1517.03</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>30 Days Warranty</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Claude - Claude Kiro API  1M</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>2491.65</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Grok - Grok API 10M Credit 1M</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>539.5700000000001</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>CapCut - CapCut Pro Team 3 Months</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>PiggyAI Premium</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>1740.2</v>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>CapCut - CapCut Pro Personal 3 Months</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>PRIVATE</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>1056.55</v>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>CapCut - CapCut Pro Team 12 Months</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>12 Months</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>22.82</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>6446.65</v>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN - NordVPN 10 Devices 3M</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>587.6</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>NordVPN - NordVPN Slot 6M</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>SHARED</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>1175.2</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Cursor Pro - Cursor Pro 2026 Credits 1M</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>2378.65</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs - ElevenLabs Redeem 100k Credits</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>1 Month</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>PremiKey Bot</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>293.8</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Full Warranty (FW)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
         </is>
       </c>
     </row>

</xml_diff>